<commit_message>
feat: refine lists, device info, params, threat alarm and message center
- Black/white list: cooperative targets, remove actions, live flight and command navigation
- Device info: archive card, deploy area select, camera seed data
- System params: control/safety/simulation groups and restore defaults
- Threat: rule priority field, sound alarm play modes and UI flash options
- Message center: device status online/offline events
- Data screen: floating object list label and refreshed prototype assets
- Flight record module and 3D map design artifacts

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/export-templates/历史事件.xlsx
+++ b/public/export-templates/历史事件.xlsx
@@ -50,8 +50,8 @@
     </font>
     <font>
       <name val="宋体"/>
-      <b val="1"/>
-      <color rgb="001E3A8A"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="宋体"/>
@@ -64,7 +64,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -74,11 +74,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001D4ED8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,10 +122,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -501,22 +496,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,55 +542,60 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>目标类型</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>发现时间</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>处置时间</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>飞手位置</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>目标型号</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>识别码</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>威胁等级</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>验证方式</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>探测设备</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>反制设备</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>处置状态</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -613,74 +614,77 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>黑飞无人机</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
           <t>2024-03-04 08:00:00</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>2024-03-04 08:00:25</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>DJI Mavic 3</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>1581F4100000</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>高危</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>人工核查</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>雷达-01 (2.4G)</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>干扰-01</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>已处置</t>
-        </is>
-      </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
+          <t>已结束</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
           <t>多源轨迹已合并</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>导出数据区（实际导出时自第 5 行起写入）</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
-    <row r="9"/>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>说明：正式导出时自第 5 行起写入数据，字段顺序与历史事件列表一致。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A7:M9"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A6:N6"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -692,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -754,185 +758,202 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>发现时间</t>
+          <t>目标类型</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>2024-03-04 08:00:00</t>
+          <t>黑飞无人机 / 飞鸟 / 其他</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>事件首次发现时间</t>
+          <t>历史事件目标类型，与列表页一致</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>处置时间</t>
+          <t>发现时间</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>2024-03-04 08:00:25 / --</t>
+          <t>2024-03-04 08:00:00</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>未完成处置时导出为 --</t>
+          <t>事件首次发现时间</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>飞手位置</t>
+          <t>处置时间</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>未定位</t>
+          <t>2024-03-04 08:00:25 / --</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>当前实现统一展示未定位</t>
+          <t>未完成处置时导出为 --</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>目标型号</t>
+          <t>飞手位置</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>DJI Mavic 3</t>
+          <t>未定位</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>识别到的目标型号</t>
+          <t>当前实现统一展示未定位</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>识别码</t>
+          <t>目标型号</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>1581F4100000 / 未解析</t>
+          <t>DJI Mavic 3</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>无人机识别码；无法识别时导出未解析</t>
+          <t>识别到的目标型号</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>威胁等级</t>
+          <t>识别码</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>高危 / 中危 / 低危 / 无危</t>
+          <t>1581F4100000 / 未解析</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>威胁评估结果，与列表展示一致</t>
+          <t>无人机识别码；无法识别时导出未解析</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>验证方式</t>
+          <t>威胁等级</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>自动识别 / 人工核查</t>
+          <t>高危 / 中危 / 低危 / 无危</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>自动识别或人工核查</t>
+          <t>威胁评估结果，与列表展示一致</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>探测设备</t>
+          <t>验证方式</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>雷达-01 (2.4G)</t>
+          <t>自动识别 / 人工核查</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>参与探测的设备</t>
+          <t>自动识别或人工核查</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>反制设备</t>
+          <t>探测设备</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>干扰-01 / --</t>
+          <t>雷达-01 (2.4G)</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>参与反制的设备名称，未执行反制时为 --</t>
+          <t>参与探测的设备</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>处置状态</t>
+          <t>反制设备</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>待处置 / 处置中 / 已处置 / 已结束</t>
+          <t>干扰-01 / --</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>事件处置状态</t>
+          <t>参与反制的设备名称，未执行反制时为 --</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
+          <t>处置状态</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>进行中 / 已结束</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>事件处置状态，与列表展示一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>多源轨迹已合并</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>补充说明；等待值守类提示不导出</t>
         </is>
@@ -1000,7 +1021,7 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>6. 模板生成时间：2026-06-29 14:01:15</t>
+          <t>6. 模板生成时间：2026-07-07 16:11:35</t>
         </is>
       </c>
     </row>

</xml_diff>